<commit_message>
Add per-sender HS breakdown and currency/incoterms consistency check
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015aKZ84k5tMpWuL4W9daZNG
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Barton_Trading_JBA20260526001.xlsx
+++ b/output/HS_Code_Summary_Barton_Trading_JBA20260526001.xlsx
@@ -7,8 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="HS Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dokumenty a poznámky" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="HS dle odesílatele" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="HS Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Dokumenty a poznámky" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,8 +38,11 @@
       <b val="1"/>
       <color rgb="00C00000"/>
     </font>
+    <font>
+      <color rgb="00C00000"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -53,6 +57,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE699"/>
       </patternFill>
     </fill>
   </fills>
@@ -74,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -87,6 +101,13 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -452,6 +473,344 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>HS kód</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Popis zboží (CZ)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Země původu (COO)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Množství</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Čistá hmotnost (kg)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Hrubá hmotnost (kg)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Hodnota (USD, FOB Ningbo)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Poznámka</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>LINHAI BILLY COMMODITY CO.,LTD — faktura 26111 (01.06.2026) — 948 ctns — house B/L …FDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>96039091</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Úklidové výrobky z plastu PP+PE – smetáček s lopatkou, smeták s násadou 120 cm, smetáček; WC sady (miska + štětka), WC štětka (tyčka + hlava); čisticí kartáč na nádobí</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>35832</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>3760</v>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>4456.9</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>11817.36</v>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>9 položek packing listu sloučeno pod jeden HS kód</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>ZHEJIANG KELIN HOME CO.,LTD — faktura KL260602 (02.06.2026) — 252 ctns — house B/L …FDC</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>39249000</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Protiskluzové podložky do vany či sprchy z PVC, různé barvy a rozměry (100% PVC)</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>6048</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>2923.2</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>3175.2</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>6804</v>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>6 položek (2 velikosti × 3 barvy)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>NINGBO AIJE HOME PRODUCTS CO.,LTD — faktura AJT2409035 (30.05.2026) — 227 ctns — house B/L …FDB</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>39211900</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Houbička melaminová NANO 4 ks/balení – čisticí houbička pro domácnost, materiál melamin</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>12024</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>100.2</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>200.4</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>2164.32</v>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>množství = balení po 4 ks</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>39249000</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Houbová drátěnka 2 ks/sada (vnější polyester/polyethylen, vnitřní houbička polyuretan)</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>7200</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>198</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>240</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>1296</v>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>množství = sady po 2 ks</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr"/>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Mezisoučet dodavatel</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr"/>
+      <c r="D9" s="4" t="n">
+        <v>19224</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>298.2</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>440.4</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>3460.32</v>
+      </c>
+      <c r="H9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>LAIZHOU LUTONG PLASTICS CO.,LTD — faktura LTP260325L (06.05.2026) — 260 ctns — house B/L …FDD</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>56090000</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Bavlněná šňůra na prádlo 15 m / 20 m (splétaná z prováků průměr 5 mm)</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>16000</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>2160</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>2290</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>9322</v>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>6 000 ks (15 m) + 10 000 ks (20 m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>CELKEM zásilka</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr"/>
+      <c r="C12" s="8" t="inlineStr"/>
+      <c r="D12" s="8" t="n">
+        <v>77104</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>9141.4</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>10362.5</v>
+      </c>
+      <c r="G12" s="8" t="n">
+        <v>31403.68</v>
+      </c>
+      <c r="H12" s="8" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Měna a Incoterms:</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Všechny 4 faktury shodně: měna USD, dodací podmínka FOB NINGBO. Všechny 4 house B/L: FREIGHT COLLECT (v souladu s FOB – námořné hradí kupující). Bez rozporu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>POZOR – preferenční věta:</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Není v žádném dokladu. Původ CN u všech položek – standardní třetizemní clo.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A10:H10"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -729,13 +1088,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:A36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -789,9 +1148,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-    </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9">
         <f>== FAKTURY (4 dodavatelé, FOB NINGBO) ===</f>
@@ -833,9 +1190,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-    </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16">
         <f>== PREFERENČNÍ VĚTA (COO) ===</f>
@@ -856,9 +1211,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr"/>
-    </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20">
         <f>== CBAM / ANTIDUMPING ===</f>
@@ -879,9 +1232,7 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr"/>
-    </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24">
         <f>== POZNÁMKY K MNOŽSTVÍ ===</f>
@@ -916,6 +1267,57 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <f>== MĚNA A INCOTERMS – KONTROLA SHODY ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Linhai 26111: USD, 'Incoterms: FOB NINGBO' ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Kelin KL260602: USD, cenový sloupec 'FOB NINGBO' ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>AIJE AJT2409035: USD, 'FOB NINGBO' ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Laizhou LTP260325L: USD, 'UNIT PRICE FOB NINGBO' ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>House B/L A–D: všechny FREIGHT COLLECT – konzistentní s FOB.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>→ Vše shodné: USD / FOB NINGBO. Žádná diskrepance. (Incoterm se dle pravidel do HS souhrnu jako sloupec neuvádí.)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>